<commit_message>
Complete first breadth samples across all 39 universities
</commit_message>
<xml_diff>
--- a/site/exports/cau-ciee-computer.xlsx
+++ b/site/exports/cau-ciee-computer.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R14692c8f22c34150"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="Rf5e59b620a1546c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Re22329ee7acf4b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R2cfb925013ff46be"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R42f9f098b3c14109"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="总览" sheetId="1" r:id="R638b87885b9c4d5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="经历" sheetId="2" r:id="R8bbccd4fcdf34bec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="导师" sheetId="3" r:id="Rc762bb8eb81d46a0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="论文" sheetId="4" r:id="R5ed53b910cf7404f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="来源" sheetId="5" r:id="R4bf1a7b6f6564da4"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -144,12 +144,12 @@
     <x:tableColumn id="1" name="姓名"/>
     <x:tableColumn id="2" name="校区"/>
     <x:tableColumn id="3" name="院系"/>
-    <x:tableColumn id="4" name="官方主页"/>
+    <x:tableColumn id="4" name="个人主页／职业网站（来源类型见说明）"/>
     <x:tableColumn id="5" name="核对日期"/>
     <x:tableColumn id="6" name="缺项与冲突"/>
     <x:tableColumn id="7" name="范围"/>
     <x:tableColumn id="8" name="主页可用性"/>
-    <x:tableColumn id="9" name="替代官方职业报道（非个人主页）"/>
+    <x:tableColumn id="9" name="替代职业资料来源（非已核个人主页）"/>
     <x:tableColumn id="10" name="所属学校ID"/>
     <x:tableColumn id="11" name="所属学校"/>
   </x:tableColumns>
@@ -417,12 +417,12 @@
     <x:col min="1" max="1" width="26" hidden="0" customWidth="1"/>
     <x:col min="2" max="2" width="26" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="26" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="26" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="55" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="26" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="55" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="55" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="26" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="26" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="55" hidden="0" customWidth="1"/>
     <x:col min="10" max="10" width="26" hidden="0" customWidth="1"/>
     <x:col min="11" max="11" width="26" hidden="0" customWidth="1"/>
   </x:cols>
@@ -438,7 +438,7 @@
         <x:v>院系</x:v>
       </x:c>
       <x:c r="D1" s="9" t="str">
-        <x:v>官方主页</x:v>
+        <x:v>个人主页／职业网站（来源类型见说明）</x:v>
       </x:c>
       <x:c r="E1" s="9" t="str">
         <x:v>核对日期</x:v>
@@ -453,7 +453,7 @@
         <x:v>主页可用性</x:v>
       </x:c>
       <x:c r="I1" s="9" t="str">
-        <x:v>替代官方职业报道（非个人主页）</x:v>
+        <x:v>替代职业资料来源（非已核个人主页）</x:v>
       </x:c>
       <x:c r="J1" s="9" t="str">
         <x:v>所属学校ID</x:v>
@@ -564,7 +564,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R4328e0615f494a8e"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R81ea2b781f0f4824"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1057,7 +1057,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf10bedb41ab04fd6"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R3da18c231dc3433d"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1254,7 +1254,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R04ae9c8996324dd4"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R950566c0f28542eb"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -1482,7 +1482,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1c9ff8163e5e479b"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R9f96337cebf34889"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>